<commit_message>
chore: Update .gitignore and modify example Excel files
- Added `Examples/bdtocb_csc_extract.xlsx` to .gitignore to prevent tracking.
- Updated `Examples/2-1bd_xml_extract.xlsx` and `Examples/bdtocb_csc_extract.xlsx` to reflect changes in their binary content.
</commit_message>
<xml_diff>
--- a/Examples/2-1bd_xml_extract.xlsx
+++ b/Examples/2-1bd_xml_extract.xlsx
@@ -1506,10 +1506,10 @@
         <v>-94.32429171798719</v>
       </c>
       <c r="L3">
-        <v>0.4009801737580754</v>
+        <v>0.4009801737580753</v>
       </c>
       <c r="M3">
-        <v>2.481617647058823E-09</v>
+        <v>2.481617647058824E-09</v>
       </c>
       <c r="N3">
         <v>6.188878676470588E-09</v>
@@ -1600,7 +1600,7 @@
         <v>-93.49260156373357</v>
       </c>
       <c r="L5">
-        <v>0.8140192299971797</v>
+        <v>0.8140192299971796</v>
       </c>
       <c r="M5">
         <v>4.890783221809485E-09</v>
@@ -1747,7 +1747,7 @@
         <v>8.373294175341841E-09</v>
       </c>
       <c r="N8">
-        <v>5.747002936849361E-09</v>
+        <v>5.74700293684936E-09</v>
       </c>
       <c r="O8">
         <v>170</v>
@@ -1782,16 +1782,16 @@
         <v>2.5</v>
       </c>
       <c r="J9">
-        <v>-23.75256986561703</v>
+        <v>-23.75256986561704</v>
       </c>
       <c r="K9">
-        <v>-23.75256986561703</v>
+        <v>-23.75256986561704</v>
       </c>
       <c r="L9">
         <v>1.677735508004749</v>
       </c>
       <c r="M9">
-        <v>9.500157496292692E-09</v>
+        <v>9.50015749629269E-09</v>
       </c>
       <c r="N9">
         <v>5.662488187778046E-09</v>
@@ -2111,10 +2111,10 @@
         <v>2.5</v>
       </c>
       <c r="J16">
-        <v>-0.5724821798156938</v>
+        <v>-0.5724821798156937</v>
       </c>
       <c r="K16">
-        <v>-0.5724821798156938</v>
+        <v>-0.5724821798156937</v>
       </c>
       <c r="L16">
         <v>3.318052600356962</v>
@@ -2214,10 +2214,10 @@
         <v>3.818818272232256</v>
       </c>
       <c r="M18">
-        <v>1.892471338898466E-08</v>
+        <v>1.892471338898465E-08</v>
       </c>
       <c r="N18">
-        <v>4.95564649582615E-09</v>
+        <v>4.955646495826151E-09</v>
       </c>
       <c r="O18">
         <v>170</v>
@@ -2883,7 +2883,7 @@
         <v>-163.051915113771</v>
       </c>
       <c r="C46">
-        <v>-38.9703430004233</v>
+        <v>-38.9703430004234</v>
       </c>
     </row>
     <row r="47">
@@ -3048,7 +3048,7 @@
         <v>-163.046919387852</v>
       </c>
       <c r="C61">
-        <v>-38.9691489932723</v>
+        <v>-38.9691489932724</v>
       </c>
     </row>
     <row r="62">
@@ -3653,7 +3653,7 @@
         <v>-163.033762815605</v>
       </c>
       <c r="C116">
-        <v>-38.9660044970375</v>
+        <v>-38.9660044970374</v>
       </c>
     </row>
     <row r="117">
@@ -3686,7 +3686,7 @@
         <v>-163.032130427265</v>
       </c>
       <c r="C119">
-        <v>-38.9656143468605</v>
+        <v>-38.9656143468606</v>
       </c>
     </row>
     <row r="120">
@@ -4324,7 +4324,7 @@
         <v>-163.045678449561</v>
       </c>
       <c r="C177">
-        <v>-38.9688524019027</v>
+        <v>-38.9688524019026</v>
       </c>
     </row>
     <row r="178">
@@ -5325,7 +5325,7 @@
         <v>-163.042765318767</v>
       </c>
       <c r="C268">
-        <v>-38.9681561469329</v>
+        <v>-38.968156146933</v>
       </c>
     </row>
     <row r="269">
@@ -5369,7 +5369,7 @@
         <v>-163.042170761904</v>
       </c>
       <c r="C272">
-        <v>-38.9680140444321</v>
+        <v>-38.9680140444322</v>
       </c>
     </row>
     <row r="273">
@@ -6249,7 +6249,7 @@
         <v>-161.386588481884</v>
       </c>
       <c r="C352">
-        <v>-38.5723203828595</v>
+        <v>-38.5723203828594</v>
       </c>
     </row>
     <row r="353">
@@ -6634,7 +6634,7 @@
         <v>-162.985209137674</v>
       </c>
       <c r="C387">
-        <v>-38.9543998895015</v>
+        <v>-38.9543998895014</v>
       </c>
     </row>
     <row r="388">
@@ -7074,7 +7074,7 @@
         <v>-163.054859388806</v>
       </c>
       <c r="C427">
-        <v>-38.9710466990455</v>
+        <v>-38.9710466990454</v>
       </c>
     </row>
     <row r="428">
@@ -7855,7 +7855,7 @@
         <v>-163.050669265174</v>
       </c>
       <c r="C498">
-        <v>-38.9700452354621</v>
+        <v>-38.9700452354622</v>
       </c>
     </row>
     <row r="499">
@@ -8317,7 +8317,7 @@
         <v>-159.762041859204</v>
       </c>
       <c r="C540">
-        <v>-38.184044421416</v>
+        <v>-38.1840444214159</v>
       </c>
     </row>
     <row r="541">
@@ -9714,7 +9714,7 @@
         <v>-163.073675170259</v>
       </c>
       <c r="C667">
-        <v>-38.9755437787425</v>
+        <v>-38.9755437787426</v>
       </c>
     </row>
     <row r="668">
@@ -9758,7 +9758,7 @@
         <v>-163.072432544911</v>
       </c>
       <c r="C671">
-        <v>-38.9752467841565</v>
+        <v>-38.9752467841566</v>
       </c>
     </row>
     <row r="672">
@@ -9978,7 +9978,7 @@
         <v>-163.075561100539</v>
       </c>
       <c r="C691">
-        <v>-38.9759945268975</v>
+        <v>-38.9759945268974</v>
       </c>
     </row>
     <row r="692">
@@ -10077,7 +10077,7 @@
         <v>-163.076006300116</v>
       </c>
       <c r="C700">
-        <v>-38.9761009321501</v>
+        <v>-38.97610093215</v>
       </c>
     </row>
     <row r="701">
@@ -10902,7 +10902,7 @@
         <v>-162.797459245584</v>
       </c>
       <c r="C775">
-        <v>-38.9095265883327</v>
+        <v>-38.9095265883326</v>
       </c>
     </row>
     <row r="776">
@@ -11342,7 +11342,7 @@
         <v>-163.072713111265</v>
       </c>
       <c r="C815">
-        <v>-38.9753138411245</v>
+        <v>-38.9753138411244</v>
       </c>
     </row>
     <row r="816">
@@ -11672,7 +11672,7 @@
         <v>-163.082872378628</v>
       </c>
       <c r="C845">
-        <v>-38.9777419642993</v>
+        <v>-38.9777419642994</v>
       </c>
     </row>
     <row r="846">
@@ -12101,7 +12101,7 @@
         <v>-163.093291618263</v>
       </c>
       <c r="C884">
-        <v>-38.9802322223383</v>
+        <v>-38.9802322223382</v>
       </c>
     </row>
     <row r="885">
@@ -12607,7 +12607,7 @@
         <v>-161.009436848568</v>
       </c>
       <c r="C930">
-        <v>-38.4821789791033</v>
+        <v>-38.4821789791032</v>
       </c>
     </row>
     <row r="931">
@@ -13223,7 +13223,7 @@
         <v>-162.959392072115</v>
       </c>
       <c r="C986">
-        <v>-38.9482294627427</v>
+        <v>-38.9482294627426</v>
       </c>
     </row>
     <row r="987">
@@ -13278,7 +13278,7 @@
         <v>-163.009992769334</v>
       </c>
       <c r="C991">
-        <v>-38.9603233196305</v>
+        <v>-38.9603233196304</v>
       </c>
     </row>
     <row r="992">
@@ -13861,7 +13861,7 @@
         <v>-163.105569870995</v>
       </c>
       <c r="C1044">
-        <v>-38.9831667951709</v>
+        <v>-38.983166795171</v>
       </c>
     </row>
     <row r="1045">
@@ -14334,7 +14334,7 @@
         <v>-163.101729750199</v>
       </c>
       <c r="C1087">
-        <v>-38.9822489842731</v>
+        <v>-38.9822489842732</v>
       </c>
     </row>
     <row r="1088">
@@ -14763,7 +14763,7 @@
         <v>-162.136294711232</v>
       </c>
       <c r="C1126">
-        <v>-38.7515044720917</v>
+        <v>-38.7515044720918</v>
       </c>
     </row>
     <row r="1127">
@@ -15093,7 +15093,7 @@
         <v>-161.877190487525</v>
       </c>
       <c r="C1156">
-        <v>-38.6895770763683</v>
+        <v>-38.6895770763682</v>
       </c>
     </row>
     <row r="1157">
@@ -15577,7 +15577,7 @@
         <v>-162.906619803547</v>
       </c>
       <c r="C1200">
-        <v>-38.935616587846</v>
+        <v>-38.9356165878459</v>
       </c>
     </row>
     <row r="1201">
@@ -15808,7 +15808,7 @@
         <v>-163.018924941197</v>
       </c>
       <c r="C1221">
-        <v>-38.9624581599419</v>
+        <v>-38.9624581599418</v>
       </c>
     </row>
     <row r="1222">
@@ -15841,7 +15841,7 @@
         <v>-163.028061866329</v>
       </c>
       <c r="C1224">
-        <v>-38.9646419374591</v>
+        <v>-38.9646419374592</v>
       </c>
     </row>
     <row r="1225">
@@ -17469,7 +17469,7 @@
         <v>-162.930589054939</v>
       </c>
       <c r="C1372">
-        <v>-38.9413453764196</v>
+        <v>-38.9413453764195</v>
       </c>
     </row>
     <row r="1373">
@@ -17821,7 +17821,7 @@
         <v>-163.076874182155</v>
       </c>
       <c r="C1404">
-        <v>-38.9763083609357</v>
+        <v>-38.9763083609356</v>
       </c>
     </row>
     <row r="1405">
@@ -17964,7 +17964,7 @@
         <v>-163.091556607654</v>
       </c>
       <c r="C1417">
-        <v>-38.9798175448503</v>
+        <v>-38.9798175448504</v>
       </c>
     </row>
     <row r="1418">
@@ -18228,7 +18228,7 @@
         <v>-163.102537659522</v>
       </c>
       <c r="C1441">
-        <v>-38.9824420792357</v>
+        <v>-38.9824420792358</v>
       </c>
     </row>
     <row r="1442">
@@ -19647,7 +19647,7 @@
         <v>-163.032246794409</v>
       </c>
       <c r="C1570">
-        <v>-38.9656421592757</v>
+        <v>-38.9656421592756</v>
       </c>
     </row>
     <row r="1571">
@@ -20098,7 +20098,7 @@
         <v>-163.121475300906</v>
       </c>
       <c r="C1611">
-        <v>-38.9869682841555</v>
+        <v>-38.9869682841554</v>
       </c>
     </row>
     <row r="1612">
@@ -20197,7 +20197,7 @@
         <v>-163.122962545256</v>
       </c>
       <c r="C1620">
-        <v>-38.987323744086</v>
+        <v>-38.9873237440859</v>
       </c>
     </row>
     <row r="1621">
@@ -20824,7 +20824,7 @@
         <v>-163.107491169269</v>
       </c>
       <c r="C1677">
-        <v>-38.9836259964792</v>
+        <v>-38.9836259964791</v>
       </c>
     </row>
     <row r="1678">
@@ -22826,7 +22826,7 @@
         <v>-163.140156980819</v>
       </c>
       <c r="C1859">
-        <v>-38.9914333128153</v>
+        <v>-38.9914333128154</v>
       </c>
     </row>
     <row r="1860">
@@ -23398,7 +23398,7 @@
         <v>-163.128717816009</v>
       </c>
       <c r="C1911">
-        <v>-38.9886992868091</v>
+        <v>-38.988699286809</v>
       </c>
     </row>
     <row r="1912">
@@ -23717,7 +23717,7 @@
         <v>-162.420119253246</v>
       </c>
       <c r="C1940">
-        <v>-38.8193401656897</v>
+        <v>-38.8193401656898</v>
       </c>
     </row>
     <row r="1941">
@@ -23893,7 +23893,7 @@
         <v>-162.826349947887</v>
       </c>
       <c r="C1956">
-        <v>-38.9164316319041</v>
+        <v>-38.9164316319042</v>
       </c>
     </row>
     <row r="1957">
@@ -24047,7 +24047,7 @@
         <v>-163.030098933777</v>
       </c>
       <c r="C1970">
-        <v>-38.9651288082641</v>
+        <v>-38.9651288082642</v>
       </c>
     </row>
     <row r="1971">
@@ -24795,7 +24795,7 @@
         <v>-163.14104394611</v>
       </c>
       <c r="C2038">
-        <v>-38.9916453026075</v>
+        <v>-38.9916453026074</v>
       </c>
     </row>
     <row r="2039">
@@ -25059,7 +25059,7 @@
         <v>-163.14312141552</v>
       </c>
       <c r="C2062">
-        <v>-38.9921418297132</v>
+        <v>-38.9921418297131</v>
       </c>
     </row>
     <row r="2063">
@@ -25389,7 +25389,7 @@
         <v>-163.136277432893</v>
       </c>
       <c r="C2092">
-        <v>-38.9905060786073</v>
+        <v>-38.9905060786072</v>
       </c>
     </row>
     <row r="2093">
@@ -25675,7 +25675,7 @@
         <v>-163.093878133944</v>
       </c>
       <c r="C2118">
-        <v>-38.9803724029503</v>
+        <v>-38.9803724029502</v>
       </c>
     </row>
     <row r="2119">
@@ -25807,7 +25807,7 @@
         <v>-162.659640294272</v>
       </c>
       <c r="C2130">
-        <v>-38.8765870684205</v>
+        <v>-38.8765870684206</v>
       </c>
     </row>
     <row r="2131">
@@ -26104,7 +26104,7 @@
         <v>-162.860113196711</v>
       </c>
       <c r="C2157">
-        <v>-38.9245012420437</v>
+        <v>-38.9245012420438</v>
       </c>
     </row>
     <row r="2158">
@@ -26357,7 +26357,7 @@
         <v>-163.087365191729</v>
       </c>
       <c r="C2180">
-        <v>-38.9788157724017</v>
+        <v>-38.9788157724018</v>
       </c>
     </row>
     <row r="2181">
@@ -26654,7 +26654,7 @@
         <v>-163.142786245511</v>
       </c>
       <c r="C2207">
-        <v>-38.9920617221585</v>
+        <v>-38.9920617221584</v>
       </c>
     </row>
     <row r="2208">
@@ -27116,7 +27116,7 @@
         <v>-163.150380139444</v>
       </c>
       <c r="C2249">
-        <v>-38.993876706368</v>
+        <v>-38.9938767063679</v>
       </c>
     </row>
     <row r="2250">
@@ -27138,7 +27138,7 @@
         <v>-163.150555818349</v>
       </c>
       <c r="C2251">
-        <v>-38.9939186946341</v>
+        <v>-38.9939186946342</v>
       </c>
     </row>
     <row r="2252">
@@ -28073,7 +28073,7 @@
         <v>-162.67170125889</v>
       </c>
       <c r="C2336">
-        <v>-38.8794697081477</v>
+        <v>-38.8794697081476</v>
       </c>
     </row>
     <row r="2337">
@@ -28414,7 +28414,7 @@
         <v>-162.99149754292</v>
       </c>
       <c r="C2367">
-        <v>-38.9559028544264</v>
+        <v>-38.9559028544263</v>
       </c>
     </row>
     <row r="2368">
@@ -28502,7 +28502,7 @@
         <v>-163.049399085412</v>
       </c>
       <c r="C2375">
-        <v>-38.9697416552131</v>
+        <v>-38.9697416552132</v>
       </c>
     </row>
     <row r="2376">
@@ -28557,7 +28557,7 @@
         <v>-163.074640518826</v>
       </c>
       <c r="C2380">
-        <v>-38.9757745025876</v>
+        <v>-38.9757745025875</v>
       </c>
     </row>
     <row r="2381">
@@ -29855,7 +29855,7 @@
         <v>-163.138169177139</v>
       </c>
       <c r="C2498">
-        <v>-38.9909582163333</v>
+        <v>-38.9909582163334</v>
       </c>
     </row>
     <row r="2499">
@@ -30053,7 +30053,7 @@
         <v>-163.125621777956</v>
       </c>
       <c r="C2516">
-        <v>-38.9879593159549</v>
+        <v>-38.987959315955</v>
       </c>
     </row>
     <row r="2517">
@@ -30603,7 +30603,7 @@
         <v>-162.999832807761</v>
       </c>
       <c r="C2566">
-        <v>-38.9578950305357</v>
+        <v>-38.9578950305356</v>
       </c>
     </row>
     <row r="2567">
@@ -30922,7 +30922,7 @@
         <v>-163.102327479138</v>
       </c>
       <c r="C2595">
-        <v>-38.9823918449181</v>
+        <v>-38.9823918449182</v>
       </c>
     </row>
     <row r="2596">
@@ -31582,7 +31582,7 @@
         <v>-163.152980119347</v>
       </c>
       <c r="C2655">
-        <v>-38.9944981164787</v>
+        <v>-38.9944981164786</v>
       </c>
     </row>
     <row r="2656">
@@ -31714,7 +31714,7 @@
         <v>-163.149095717925</v>
       </c>
       <c r="C2667">
-        <v>-38.9935697222573</v>
+        <v>-38.9935697222574</v>
       </c>
     </row>
     <row r="2668">
@@ -32000,7 +32000,7 @@
         <v>-163.144078397148</v>
       </c>
       <c r="C2693">
-        <v>-38.9923705538117</v>
+        <v>-38.9923705538116</v>
       </c>
     </row>
     <row r="2694">
@@ -32055,7 +32055,7 @@
         <v>-163.142321978709</v>
       </c>
       <c r="C2698">
-        <v>-38.9919507597297</v>
+        <v>-38.9919507597296</v>
       </c>
     </row>
     <row r="2699">
@@ -32517,7 +32517,7 @@
         <v>-162.991808041567</v>
       </c>
       <c r="C2740">
-        <v>-38.9559770653841</v>
+        <v>-38.9559770653842</v>
       </c>
     </row>
     <row r="2741">
@@ -32759,7 +32759,7 @@
         <v>-163.0571946206</v>
       </c>
       <c r="C2762">
-        <v>-38.9716048328393</v>
+        <v>-38.9716048328394</v>
       </c>
     </row>
     <row r="2763">
@@ -33089,7 +33089,7 @@
         <v>-163.125880261206</v>
       </c>
       <c r="C2792">
-        <v>-38.9880210949345</v>
+        <v>-38.9880210949344</v>
       </c>
     </row>
     <row r="2793">
@@ -33320,7 +33320,7 @@
         <v>-163.136254947337</v>
       </c>
       <c r="C2813">
-        <v>-38.9905007044305</v>
+        <v>-38.9905007044304</v>
       </c>
     </row>
     <row r="2814">
@@ -33430,7 +33430,7 @@
         <v>-163.141724561786</v>
       </c>
       <c r="C2823">
-        <v>-38.9918079736581</v>
+        <v>-38.9918079736582</v>
       </c>
     </row>
     <row r="2824">
@@ -33496,7 +33496,7 @@
         <v>-163.142673752937</v>
       </c>
       <c r="C2829">
-        <v>-38.992034835788</v>
+        <v>-38.9920348357879</v>
       </c>
     </row>
     <row r="2830">
@@ -34563,7 +34563,7 @@
         <v>-163.110071479839</v>
       </c>
       <c r="C2926">
-        <v>-38.9842427055065</v>
+        <v>-38.9842427055066</v>
       </c>
     </row>
     <row r="2927">
@@ -34772,7 +34772,7 @@
         <v>-163.102034581261</v>
       </c>
       <c r="C2945">
-        <v>-38.9823218406457</v>
+        <v>-38.9823218406456</v>
       </c>
     </row>
     <row r="2946">
@@ -35663,7 +35663,7 @@
         <v>-163.148183281614</v>
       </c>
       <c r="C3026">
-        <v>-38.9933516447453</v>
+        <v>-38.9933516447452</v>
       </c>
     </row>
     <row r="3027">
@@ -35861,7 +35861,7 @@
         <v>-163.151158557756</v>
       </c>
       <c r="C3044">
-        <v>-38.9940627528097</v>
+        <v>-38.9940627528098</v>
       </c>
     </row>
     <row r="3045">
@@ -37192,7 +37192,7 @@
         <v>-163.138444013309</v>
       </c>
       <c r="C3165">
-        <v>-38.9910239037545</v>
+        <v>-38.9910239037544</v>
       </c>
     </row>
     <row r="3166">
@@ -38072,7 +38072,7 @@
         <v>-163.153554144384</v>
       </c>
       <c r="C3245">
-        <v>-38.9946353117553</v>
+        <v>-38.9946353117552</v>
       </c>
     </row>
     <row r="3246">
@@ -38567,7 +38567,7 @@
         <v>-163.158839336395</v>
       </c>
       <c r="C3290">
-        <v>-38.9958985029625</v>
+        <v>-38.9958985029624</v>
       </c>
     </row>
     <row r="3291">
@@ -39062,7 +39062,7 @@
         <v>-163.188443861432</v>
       </c>
       <c r="C3335">
-        <v>-39.002974154262</v>
+        <v>-39.0029741542619</v>
       </c>
     </row>
     <row r="3336">
@@ -39337,7 +39337,7 @@
         <v>-163.169467605022</v>
       </c>
       <c r="C3360">
-        <v>-38.9984387201295</v>
+        <v>-38.9984387201296</v>
       </c>
     </row>
     <row r="3361">
@@ -40360,7 +40360,7 @@
         <v>-163.175214217447</v>
       </c>
       <c r="C3453">
-        <v>-38.9998121934625</v>
+        <v>-38.9998121934624</v>
       </c>
     </row>
     <row r="3454">
@@ -41042,7 +41042,7 @@
         <v>-163.171716544319</v>
       </c>
       <c r="C3515">
-        <v>-38.9989762295217</v>
+        <v>-38.9989762295218</v>
       </c>
     </row>
     <row r="3516">
@@ -41229,7 +41229,7 @@
         <v>-163.197385789131</v>
       </c>
       <c r="C3532">
-        <v>-39.0051113262741</v>
+        <v>-39.005111326274</v>
       </c>
     </row>
     <row r="3533">
@@ -41350,7 +41350,7 @@
         <v>-163.216611312966</v>
       </c>
       <c r="C3543">
-        <v>-39.0097063367509</v>
+        <v>-39.0097063367508</v>
       </c>
     </row>
     <row r="3544">
@@ -41482,7 +41482,7 @@
         <v>-163.187882015138</v>
       </c>
       <c r="C3555">
-        <v>-39.0028398697749</v>
+        <v>-39.002839869775</v>
       </c>
     </row>
     <row r="3556">
@@ -41537,7 +41537,7 @@
         <v>-163.177797105372</v>
       </c>
       <c r="C3560">
-        <v>-39.0004295184925</v>
+        <v>-39.0004295184924</v>
       </c>
     </row>
     <row r="3561">
@@ -41823,7 +41823,7 @@
         <v>-163.169634759105</v>
       </c>
       <c r="C3586">
-        <v>-38.9984786709141</v>
+        <v>-38.9984786709142</v>
       </c>
     </row>
     <row r="3587">
@@ -42274,7 +42274,7 @@
         <v>-163.166841628251</v>
       </c>
       <c r="C3627">
-        <v>-38.9978110966183</v>
+        <v>-38.9978110966184</v>
       </c>
     </row>
     <row r="3628">
@@ -43231,7 +43231,7 @@
         <v>-163.160153366511</v>
       </c>
       <c r="C3714">
-        <v>-38.9962125636977</v>
+        <v>-38.9962125636976</v>
       </c>
     </row>
     <row r="3715">
@@ -44199,7 +44199,7 @@
         <v>-163.180201581095</v>
       </c>
       <c r="C3802">
-        <v>-39.0010042019825</v>
+        <v>-39.0010042019824</v>
       </c>
     </row>
     <row r="3803">
@@ -44397,7 +44397,7 @@
         <v>-163.186960443527</v>
       </c>
       <c r="C3820">
-        <v>-39.0026196088735</v>
+        <v>-39.0026196088734</v>
       </c>
     </row>
     <row r="3821">
@@ -44408,7 +44408,7 @@
         <v>-163.186736581416</v>
       </c>
       <c r="C3821">
-        <v>-39.0025661045449</v>
+        <v>-39.002566104545</v>
       </c>
     </row>
     <row r="3822">
@@ -45321,7 +45321,7 @@
         <v>-163.192420713184</v>
       </c>
       <c r="C3904">
-        <v>-39.0039246446425</v>
+        <v>-39.0039246446426</v>
       </c>
     </row>
     <row r="3905">
@@ -45607,7 +45607,7 @@
         <v>-163.200756292691</v>
       </c>
       <c r="C3930">
-        <v>-39.0059168959588</v>
+        <v>-39.0059168959587</v>
       </c>
     </row>
     <row r="3931">
@@ -45959,7 +45959,7 @@
         <v>-163.206964176364</v>
       </c>
       <c r="C3962">
-        <v>-39.0074006157659</v>
+        <v>-39.0074006157658</v>
       </c>
     </row>
     <row r="3963">
@@ -46168,7 +46168,7 @@
         <v>-163.19621179134</v>
       </c>
       <c r="C3981">
-        <v>-39.0048307340679</v>
+        <v>-39.0048307340678</v>
       </c>
     </row>
     <row r="3982">
@@ -46388,7 +46388,7 @@
         <v>-163.202402232504</v>
       </c>
       <c r="C4001">
-        <v>-39.0063102850153</v>
+        <v>-39.0063102850152</v>
       </c>
     </row>
     <row r="4002">
@@ -46520,7 +46520,7 @@
         <v>-163.204149436709</v>
       </c>
       <c r="C4013">
-        <v>-39.0067278768425</v>
+        <v>-39.0067278768426</v>
       </c>
     </row>
     <row r="4014">
@@ -46674,7 +46674,7 @@
         <v>-163.20154310269</v>
       </c>
       <c r="C4027">
-        <v>-39.0061049480616</v>
+        <v>-39.0061049480615</v>
       </c>
     </row>
     <row r="4028">
@@ -46773,7 +46773,7 @@
         <v>-163.197147743034</v>
       </c>
       <c r="C4036">
-        <v>-39.0050544318915</v>
+        <v>-39.0050544318914</v>
       </c>
     </row>
     <row r="4037">
@@ -47433,7 +47433,7 @@
         <v>-163.201908278758</v>
       </c>
       <c r="C4096">
-        <v>-39.0061922272365</v>
+        <v>-39.0061922272366</v>
       </c>
     </row>
     <row r="4097">
@@ -48236,7 +48236,7 @@
         <v>-163.205114423123</v>
       </c>
       <c r="C4169">
-        <v>-39.0069585141307</v>
+        <v>-39.0069585141306</v>
       </c>
     </row>
     <row r="4170">
@@ -48665,7 +48665,7 @@
         <v>-163.215427499704</v>
       </c>
       <c r="C4208">
-        <v>-39.0094233985908</v>
+        <v>-39.0094233985907</v>
       </c>
     </row>
     <row r="4209">
@@ -48929,7 +48929,7 @@
         <v>-163.215016340315</v>
       </c>
       <c r="C4232">
-        <v>-39.0093251291385</v>
+        <v>-39.0093251291384</v>
       </c>
     </row>
     <row r="4233">

</xml_diff>